<commit_message>
diff analysis: add a column dictionary sheet; ignore Excel lock files
</commit_message>
<xml_diff>
--- a/manifest/fl-election-day-diffs.xlsx
+++ b/manifest/fl-election-day-diffs.xlsx
@@ -14,7 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Numbers" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notable and rare" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uncategorized sample" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'By county'!$A$1:$Z$51</definedName>
@@ -128,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -157,6 +158,8 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -16747,6 +16750,491 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="96" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>What every column means</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="C2" s="18" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>By county</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Florida county. Only counties with at least one genuinely edited page appear; those whose site was replaced or emptied are on 'Site replaced or empty'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>By county</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>Pages changed</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>How many of this county's captured pages changed at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>By county</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>Pages captured</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>How many of the 5 page types this county publishes (from the manifest). 4/5 means one type is a recorded gap, not a failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>By county</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>% of pages changed</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Pages changed ÷ pages captured. Lets a small county that changed everything rank against a big one that changed one page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>By county</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Lines changed</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Added + removed lines of page.txt. THE unduplicated total — use this, not the sum of the category columns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>By county</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Lines added / removed</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Direction of the change. Heavy removal with light addition usually means content was retired (early voting ending); the reverse means new material was published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>By county</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Page types changed</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Which of homepage / elections / polling / early_voting / results moved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>By county</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>&lt;category columns&gt;</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Lines in this county matching that category. A line can match several categories, so these sum to MORE than 'Lines changed'. Shaded darker green the higher the count, to read across counties at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>By category</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Line hits</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Total matching lines across every county.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>By category</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Counties affected</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>How many distinct counties had at least one line in this category — the better measure of how WIDESPREAD a behaviour is, where 'Line hits' measures VOLUME and can be driven by one verbose county.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>By category</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>% of 67 counties</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Counties affected ÷ 67.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>By category</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>Share of all categorized hits</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>This category's line hits ÷ all category hits. Shows the shape of election-day activity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>By category</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>Example</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>One real changed line, so the category is not taken on trust.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>By page type</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>Files changed</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Pages of this type that changed, across all counties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>By page type</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>Top categories</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>The four categories with most lines for this page type — what this kind of page is FOR on election day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Site replaced or empty</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>What happened</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>'replaced by election-night page' = the county swapped its whole site for a minimal static page. 'served empty HTML' = the URL returned no content. 'capture path changed' = the plain/headless fetch path differed between runs, so the two sides are NOT comparable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Site replaced or empty</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Bytes before / after</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Response size either side. This is what identifies a replacement: Calhoun's polling page went 202,198 → 49 bytes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Site replaced or empty</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>% of bytes retained</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>After ÷ before. Under 25% means replaced, not edited.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Site replaced or empty</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>HTTP status</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Status before → after. 200 → 404 is the tell that the old URL no longer exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Site replaced or empty</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Render mode</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>plain → headless (or the reverse). A flip changes how much of the page is captured, which is why those rows are excluded from the content counts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>'changed' = the same sentence appears on both sides with only its digits different, so before/after are directly comparable. 'new' = a figure that appears only in the added text and has no prior value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>Measure (digits masked)</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>The sentence with its numbers replaced by N — this is the key the before/after pairing is done on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>Before / After</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>The actual lines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>After − before, filled only where each side carried exactly one comparable number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Notable and rare</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>Counties with it</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>How many counties showed this category at all. Rows are limited to categories confined to 5 or fewer counties — the unusual behaviour, as opposed to what everyone did.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Uncategorized sample</t>
+        </is>
+      </c>
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>Changed line</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>A changed line that matched no category. Shown so the keyword lists can be improved; a large count here means the categories are incomplete, NOT that nothing happened.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -16767,7 +17255,7 @@
           <t>Comparison</t>
         </is>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="20" t="inlineStr">
         <is>
           <t>50a50696  2026-08-06  snapshot run 2026-08-06T10:26:53Z (314 targets)
     →  working tree (fresh capture)</t>
@@ -16780,7 +17268,7 @@
           <t>Unit of measure</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>One line of page.txt. A file that changed in three places contributes three lines.</t>
         </is>
@@ -16792,7 +17280,7 @@
           <t>Artifact used</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>page.txt only — the visible-text artifact. page.html carries the same change plus markup, so counting both would double-count.</t>
         </is>
@@ -16804,7 +17292,7 @@
           <t>Categories overlap</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>A line can match several categories, so category columns sum to MORE than 'Lines changed'. Use 'Lines changed' for totals and the category columns for shape.</t>
         </is>
@@ -16816,7 +17304,7 @@
           <t>Noise floor</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>Two back-to-back captures of these same 314 targets produced a 0-line diff, so every line counted here is a real content change, not capture jitter.</t>
         </is>
@@ -16828,7 +17316,7 @@
           <t>Numbers that moved</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>Recorded only where the same sentence appears on both sides of the diff with just its digits changed — that pairing is what makes before/after comparable.</t>
         </is>
@@ -16840,7 +17328,7 @@
           <t>Uncategorized</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>Shown so the keyword lists can be improved. A high count there means the categories are missing something, not that nothing happened.</t>
         </is>
@@ -16852,7 +17340,7 @@
           <t>Regenerate</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>python scripts/analyze_diffs.py --from &lt;rev&gt; [--to &lt;rev&gt;]</t>
         </is>

</xml_diff>

<commit_message>
diff analysis: correct how the category columns reconcile
</commit_message>
<xml_diff>
--- a/manifest/fl-election-day-diffs.xlsx
+++ b/manifest/fl-election-day-diffs.xlsx
@@ -16914,7 +16914,7 @@
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Lines in this county matching that category. A line can match several categories, so these sum to MORE than 'Lines changed'. Shaded darker green the higher the count, to read across counties at a glance.</t>
+          <t>Lines in this county matching that category. These do NOT sum to 'Lines changed' and are not a partition of it: a line matching two categories is counted twice, and a line matching none is not counted at all. The second dominates — Escambia changed 1,089 lines, 480 matched nothing, so its categories total 408. Shaded darker green the higher the count, to compare across counties at a glance.</t>
         </is>
       </c>
     </row>
@@ -17289,12 +17289,12 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Categories overlap</t>
+          <t>Categories do not sum</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>A line can match several categories, so category columns sum to MORE than 'Lines changed'. Use 'Lines changed' for totals and the category columns for shape.</t>
+          <t>The category columns are not a partition of 'Lines changed'. A line matching two categories is counted twice; a line matching none is not counted at all. Across this run: 3,791 lines changed, 1,661 category hits, 1,368 lines matched nothing. Use 'Lines changed' for magnitude, categories for shape.</t>
         </is>
       </c>
     </row>

</xml_diff>